<commit_message>
Leva 1: operação, frequências do plano de controle pelo risco, com registro resumido por noite
- Produção, pizzaria: K4 e K7 conferidos a cada hora do pico, com a
  pior leitura (K4) e a menor temperatura (K7) registradas na noite; K5
  com 20 pedidos conferidos na saída durante o pico; K6 acompanhada no
  sistema durante a noite, com a maior espera registrada no fechamento.
  Exemplo do campo Frequência no módulo 3 com o K7 novo.
- Produção, indústria: K2, K4, K5 e K7 dizem o que a folha ou o romaneio
  registra por lote.
- Totais sem mudança (56, 6 fora, 1 sem reação; indústria 40, 5, 1).
- Ficha: P15 corrigida; N31 nova; regra N31 em PROIBIDO (Produção).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Producao/Producao-modelo.xlsx
+++ b/Producao/Producao-modelo.xlsx
@@ -163,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="471">
   <si>
     <t xml:space="preserve">Controle de produção e de serviço — Como usar esta planilha</t>
   </si>
@@ -972,13 +972,13 @@
     <t xml:space="preserve">Assar</t>
   </si>
   <si>
-    <t xml:space="preserve">Temperatura do forno</t>
+    <t xml:space="preserve">Temperatura do forno no pico: a pior leitura da noite</t>
   </si>
   <si>
     <t xml:space="preserve">Termômetro do forno, no pico do turno</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma vez por noite, no pico</t>
+    <t xml:space="preserve">A cada hora do pico; registra-se a leitura fora da faixa ou, com todas dentro, a mais afastada de 300 °C</t>
   </si>
   <si>
     <t xml:space="preserve">Pizzaiolo do turno · Registro de regulagem do forno</t>
@@ -999,7 +999,7 @@
     <t xml:space="preserve">Conferência da pizza com a etiqueta, na saída, antes de o pedido sair</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma amostra de 20 pedidos por noite, somada no fechamento</t>
+    <t xml:space="preserve">20 pedidos por noite, conferidos na saída durante o pico; o fechamento registra quantos tinham a rubrica</t>
   </si>
   <si>
     <t xml:space="preserve">Quem embala · Etiqueta rubricada</t>
@@ -1020,7 +1020,7 @@
     <t xml:space="preserve">Horários de pronto e de saída, no sistema de pedidos</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma vez por noite: a maior espera, lida no fechamento</t>
+    <t xml:space="preserve">Acompanhada no sistema durante a noite; a maior espera é registrada no fechamento</t>
   </si>
   <si>
     <t xml:space="preserve">Líder da expedição · Sistema de pedidos</t>
@@ -1029,13 +1029,13 @@
     <t xml:space="preserve">Priorizar a saída. Acima de 15 minutos, refazer a pizza.</t>
   </si>
   <si>
-    <t xml:space="preserve">Temperatura da pizza na saída</t>
+    <t xml:space="preserve">Menor temperatura da pizza na saída, na noite</t>
   </si>
   <si>
     <t xml:space="preserve">Termômetro de espeto, no centro da pizza</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma pizza por noite, no pico</t>
+    <t xml:space="preserve">Três pizzas por hora no pico; registra-se a menor temperatura da noite</t>
   </si>
   <si>
     <t xml:space="preserve">Líder da expedição · Planilha da expedição</t>
@@ -1308,7 +1308,7 @@
     <t xml:space="preserve">Leitura no painel da extrusora</t>
   </si>
   <si>
-    <t xml:space="preserve">A cada duas horas</t>
+    <t xml:space="preserve">A cada duas horas; a folha registra, por lote, a leitura mais afastada de 190 °C</t>
   </si>
   <si>
     <t xml:space="preserve">Operador · Folha de processo</t>
@@ -1341,6 +1341,9 @@
     <t xml:space="preserve">Trena calibrada TR-03</t>
   </si>
   <si>
+    <t xml:space="preserve">Cada bobina; a folha registra, por lote, a largura mais afastada de 600 mm</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ajustar as guias e segregar a bobina.</t>
   </si>
   <si>
@@ -1353,6 +1356,9 @@
     <t xml:space="preserve">Exame visual, com o padrão de defeitos do posto</t>
   </si>
   <si>
+    <t xml:space="preserve">Cada bobina; a folha registra, por lote, se todas as bobinas estão conformes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Segregar a bobina e procurar a origem: filtro, matriz ou resina.</t>
   </si>
   <si>
@@ -1384,6 +1390,9 @@
   </si>
   <si>
     <t xml:space="preserve">Conferência da etiqueta com a folha de processo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada bobina; o romaneio registra, por lote, se todas as etiquetas conferem</t>
   </si>
   <si>
     <t xml:space="preserve">Expedição · Romaneio</t>
@@ -2227,11 +2236,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="93060251"/>
-        <c:axId val="87982215"/>
+        <c:axId val="27791634"/>
+        <c:axId val="83319045"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="93060251"/>
+        <c:axId val="27791634"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -2263,7 +2272,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87982215"/>
+        <c:crossAx val="83319045"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2271,7 +2280,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87982215"/>
+        <c:axId val="83319045"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -2312,7 +2321,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93060251"/>
+        <c:crossAx val="27791634"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="0.25"/>
@@ -11955,7 +11964,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="10" t="s">
         <v>99</v>
       </c>
@@ -11990,7 +11999,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="10" t="s">
         <v>100</v>
       </c>
@@ -12023,7 +12032,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="10" t="s">
         <v>101</v>
       </c>
@@ -12056,7 +12065,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="10" t="s">
         <v>102</v>
       </c>
@@ -15137,7 +15146,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="10" t="s">
         <v>97</v>
       </c>
@@ -15207,7 +15216,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="10" t="s">
         <v>99</v>
       </c>
@@ -15233,24 +15242,24 @@
         <v>391</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>382</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="10" t="s">
         <v>100</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D17" s="32" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E17" s="33" t="s">
         <v>255</v>
@@ -15261,16 +15270,16 @@
         <v>263</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="K17" s="7" t="s">
         <v>382</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15278,10 +15287,10 @@
         <v>101</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E18" s="33" t="s">
         <v>255</v>
@@ -15291,30 +15300,30 @@
       </c>
       <c r="G18" s="34"/>
       <c r="H18" s="33" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="66.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="10" t="s">
         <v>102</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="D19" s="32" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E19" s="33" t="s">
         <v>255</v>
@@ -15325,16 +15334,16 @@
         <v>263</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>387</v>
+        <v>409</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15512,7 +15521,7 @@
         <v>100</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D27" s="7"/>
       <c r="E27" s="28" t="n">
@@ -15544,7 +15553,7 @@
         <v>101</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D28" s="7"/>
       <c r="E28" s="28" t="n">
@@ -15576,7 +15585,7 @@
         <v>102</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="28" t="n">
@@ -15654,7 +15663,7 @@
         <v>46517</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D33" s="39" t="s">
         <v>372</v>
@@ -15686,7 +15695,7 @@
         <v>46517</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D34" s="39" t="s">
         <v>379</v>
@@ -15718,7 +15727,7 @@
         <v>46517</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D35" s="39" t="s">
         <v>384</v>
@@ -15750,7 +15759,7 @@
         <v>46517</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="D36" s="39" t="s">
         <v>384</v>
@@ -15782,7 +15791,7 @@
         <v>46517</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D37" s="39" t="s">
         <v>389</v>
@@ -15814,10 +15823,10 @@
         <v>46517</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D38" s="39" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E38" s="33" t="s">
         <v>100</v>
@@ -15846,10 +15855,10 @@
         <v>46517</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D39" s="39" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E39" s="33" t="s">
         <v>101</v>
@@ -15878,10 +15887,10 @@
         <v>46517</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D40" s="39" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E40" s="33" t="s">
         <v>102</v>
@@ -15910,7 +15919,7 @@
         <v>46518</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D41" s="39" t="s">
         <v>372</v>
@@ -15942,7 +15951,7 @@
         <v>46518</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D42" s="39" t="s">
         <v>379</v>
@@ -15974,7 +15983,7 @@
         <v>46518</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="D43" s="39" t="s">
         <v>384</v>
@@ -16006,7 +16015,7 @@
         <v>46518</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="D44" s="39" t="s">
         <v>384</v>
@@ -16038,7 +16047,7 @@
         <v>46518</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D45" s="39" t="s">
         <v>389</v>
@@ -16070,10 +16079,10 @@
         <v>46518</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D46" s="39" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E46" s="33" t="s">
         <v>100</v>
@@ -16087,14 +16096,14 @@
         <v/>
       </c>
       <c r="H46" s="34" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="I46" s="22" t="str">
         <f aca="false">IF(AND(F46="",G46=""),IF(H46="","Falta o resultado",IF(H46="Sim","Dentro","Fora")),IF(H46="","Falta o valor",IF(AND(OR(F46="",H46&gt;=F46),OR(G46="",H46&lt;=G46)),"Dentro","Fora")))</f>
         <v>Fora</v>
       </c>
       <c r="J46" s="7" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
@@ -16104,10 +16113,10 @@
         <v>46518</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D47" s="39" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E47" s="33" t="s">
         <v>101</v>
@@ -16136,10 +16145,10 @@
         <v>46518</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E48" s="33" t="s">
         <v>102</v>
@@ -16168,7 +16177,7 @@
         <v>46519</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D49" s="39" t="s">
         <v>372</v>
@@ -16200,7 +16209,7 @@
         <v>46519</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D50" s="39" t="s">
         <v>379</v>
@@ -16224,7 +16233,7 @@
         <v>Fora</v>
       </c>
       <c r="J50" s="7" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="K50" s="7"/>
       <c r="L50" s="7"/>
@@ -16234,7 +16243,7 @@
         <v>46519</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="D51" s="39" t="s">
         <v>384</v>
@@ -16258,7 +16267,7 @@
         <v>Fora</v>
       </c>
       <c r="J51" s="7" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="K51" s="7"/>
       <c r="L51" s="7"/>
@@ -16268,7 +16277,7 @@
         <v>46519</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="D52" s="39" t="s">
         <v>384</v>
@@ -16300,7 +16309,7 @@
         <v>46519</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D53" s="39" t="s">
         <v>389</v>
@@ -16332,10 +16341,10 @@
         <v>46519</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D54" s="39" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E54" s="33" t="s">
         <v>100</v>
@@ -16364,10 +16373,10 @@
         <v>46519</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D55" s="39" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E55" s="33" t="s">
         <v>101</v>
@@ -16396,10 +16405,10 @@
         <v>46519</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D56" s="39" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E56" s="33" t="s">
         <v>102</v>
@@ -16428,7 +16437,7 @@
         <v>46520</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D57" s="39" t="s">
         <v>372</v>
@@ -16460,7 +16469,7 @@
         <v>46520</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D58" s="39" t="s">
         <v>379</v>
@@ -16492,7 +16501,7 @@
         <v>46520</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="D59" s="39" t="s">
         <v>384</v>
@@ -16524,7 +16533,7 @@
         <v>46520</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D60" s="39" t="s">
         <v>384</v>
@@ -16556,7 +16565,7 @@
         <v>46520</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D61" s="39" t="s">
         <v>389</v>
@@ -16588,10 +16597,10 @@
         <v>46520</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D62" s="39" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E62" s="33" t="s">
         <v>100</v>
@@ -16620,10 +16629,10 @@
         <v>46520</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D63" s="39" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E63" s="33" t="s">
         <v>101</v>
@@ -16652,10 +16661,10 @@
         <v>46520</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D64" s="39" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E64" s="33" t="s">
         <v>102</v>
@@ -16669,7 +16678,7 @@
         <v/>
       </c>
       <c r="H64" s="34" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="I64" s="22" t="str">
         <f aca="false">IF(AND(F64="",G64=""),IF(H64="","Falta o resultado",IF(H64="Sim","Dentro","Fora")),IF(H64="","Falta o valor",IF(AND(OR(F64="",H64&gt;=F64),OR(G64="",H64&lt;=G64)),"Dentro","Fora")))</f>
@@ -16684,7 +16693,7 @@
         <v>46521</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D65" s="39" t="s">
         <v>372</v>
@@ -16716,7 +16725,7 @@
         <v>46521</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D66" s="39" t="s">
         <v>379</v>
@@ -16748,7 +16757,7 @@
         <v>46521</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="D67" s="39" t="s">
         <v>384</v>
@@ -16772,7 +16781,7 @@
         <v>Fora</v>
       </c>
       <c r="J67" s="7" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
@@ -16782,7 +16791,7 @@
         <v>46521</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="D68" s="39" t="s">
         <v>384</v>
@@ -16814,7 +16823,7 @@
         <v>46521</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D69" s="39" t="s">
         <v>389</v>
@@ -16846,10 +16855,10 @@
         <v>46521</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D70" s="39" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E70" s="33" t="s">
         <v>100</v>
@@ -16878,10 +16887,10 @@
         <v>46521</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D71" s="39" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E71" s="33" t="s">
         <v>101</v>
@@ -16910,10 +16919,10 @@
         <v>46521</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D72" s="39" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="E72" s="33" t="s">
         <v>102</v>
@@ -16985,20 +16994,20 @@
         <v>371</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E76" s="7" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="F76" s="7"/>
       <c r="G76" s="7"/>
       <c r="H76" s="7"/>
       <c r="I76" s="7" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="J76" s="7"/>
       <c r="K76" s="7" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="L76" s="7"/>
     </row>
@@ -17010,20 +17019,20 @@
         <v>378</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="F77" s="7"/>
       <c r="G77" s="7"/>
       <c r="H77" s="7"/>
       <c r="I77" s="7" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="J77" s="7"/>
       <c r="K77" s="7" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="L77" s="7"/>
     </row>
@@ -17032,23 +17041,23 @@
         <v>3</v>
       </c>
       <c r="C78" s="32" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D78" s="7" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="F78" s="7"/>
       <c r="G78" s="7"/>
       <c r="H78" s="7"/>
       <c r="I78" s="7" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="J78" s="7"/>
       <c r="K78" s="7" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="L78" s="7"/>
     </row>
@@ -17057,23 +17066,23 @@
         <v>4</v>
       </c>
       <c r="C79" s="32" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="F79" s="7"/>
       <c r="G79" s="7"/>
       <c r="H79" s="7"/>
       <c r="I79" s="7" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="J79" s="7"/>
       <c r="K79" s="7" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="L79" s="7"/>
     </row>
@@ -17082,23 +17091,23 @@
         <v>5</v>
       </c>
       <c r="C80" s="32" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="E80" s="7" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="F80" s="7"/>
       <c r="G80" s="7"/>
       <c r="H80" s="7"/>
       <c r="I80" s="7" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="J80" s="7"/>
       <c r="K80" s="7" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="L80" s="7"/>
     </row>
@@ -17147,22 +17156,22 @@
         <v>1</v>
       </c>
       <c r="C84" s="32" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="D84" s="7" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="E84" s="33" t="s">
         <v>347</v>
       </c>
       <c r="F84" s="33"/>
       <c r="G84" s="7" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="H84" s="7"/>
       <c r="I84" s="7"/>
       <c r="J84" s="7" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
@@ -17172,17 +17181,17 @@
         <v>2</v>
       </c>
       <c r="C85" s="32" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="E85" s="33" t="s">
         <v>347</v>
       </c>
       <c r="F85" s="33"/>
       <c r="G85" s="7" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="H85" s="7"/>
       <c r="I85" s="7"/>
@@ -17195,17 +17204,17 @@
         <v>3</v>
       </c>
       <c r="C86" s="32" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="D86" s="7" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="E86" s="33" t="s">
         <v>351</v>
       </c>
       <c r="F86" s="33"/>
       <c r="G86" s="7" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="H86" s="7"/>
       <c r="I86" s="7"/>
@@ -17260,17 +17269,17 @@
         <v>46510</v>
       </c>
       <c r="C90" s="32" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="D90" s="7" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="E90" s="7"/>
       <c r="F90" s="7"/>
       <c r="G90" s="7"/>
       <c r="H90" s="7"/>
       <c r="I90" s="7" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="J90" s="7"/>
       <c r="K90" s="7"/>
@@ -17284,22 +17293,22 @@
         <v>46521</v>
       </c>
       <c r="C91" s="32" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D91" s="7" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="F91" s="7"/>
       <c r="G91" s="7"/>
       <c r="H91" s="7"/>
       <c r="I91" s="7" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="J91" s="7" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="K91" s="7"/>
       <c r="L91" s="13" t="str">

</xml_diff>